<commit_message>
feat(hedon): custom gallery order for Hedonist DGR 2026
- GaleriaCasco accepts a custom view order and labels.
- DGR 2026 shows three-quarter, the "-front" file (a rear three-quarter,
  labeled as such), side and back, in the showcase and its PDP.
- Catalogo Master: DGR now uses the hedonist-dgr-black-2026 photos.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Master_Lhopital-moto.xlsx
+++ b/Catalogo_Master_Lhopital-moto.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\lhopital-moto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{41F36728-6D8C-41B7-A9E0-BE0AA22CECD7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D9AF4A5-2B3A-466A-B457-95BF9A886080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -3758,9 +3758,6 @@
     <t>edenist-two-face-three-quarter</t>
   </si>
   <si>
-    <t>hedonist-dgr-2026-three-quarter</t>
-  </si>
-  <si>
     <t>HED-ASH-M-DOT</t>
   </si>
   <si>
@@ -3768,6 +3765,9 @@
   </si>
   <si>
     <t>EDE-TWF-S-NTA</t>
+  </si>
+  <si>
+    <t>hedonist-dgr-black-2026-three-quarter</t>
   </si>
 </sst>
 </file>
@@ -13836,10 +13836,10 @@
     </row>
     <row r="3" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
+        <v>1235</v>
+      </c>
+      <c r="B3" t="s">
         <v>1236</v>
-      </c>
-      <c r="B3" t="s">
-        <v>1237</v>
       </c>
       <c r="C3" t="s">
         <v>19</v>
@@ -13921,7 +13921,7 @@
     </row>
     <row r="5" spans="1:17" x14ac:dyDescent="0.45">
       <c r="A5" t="s">
-        <v>1238</v>
+        <v>1237</v>
       </c>
       <c r="B5" t="s">
         <v>1230</v>
@@ -13948,7 +13948,7 @@
         <v>1231</v>
       </c>
       <c r="J5" t="s">
-        <v>24</v>
+        <v>1231</v>
       </c>
       <c r="K5" s="16" t="s">
         <v>1228</v>
@@ -13998,7 +13998,7 @@
         <v>25</v>
       </c>
       <c r="N6" t="s">
-        <v>1235</v>
+        <v>1238</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
data(catalogo): precio de Tees a $400 en el Excel maestro
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Catalogo_Master_Lhopital-moto.xlsx
+++ b/Catalogo_Master_Lhopital-moto.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\dev\lhopital-moto\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D9AF4A5-2B3A-466A-B457-95BF9A886080}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F365A01F-AD96-491D-9D12-969FCE8F7852}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="21795" windowHeight="12975" firstSheet="5" activeTab="8" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="LÉEME" sheetId="1" r:id="rId1"/>
@@ -18278,11 +18278,11 @@
       <c r="E2" t="s">
         <v>29</v>
       </c>
-      <c r="F2">
-        <v>850</v>
+      <c r="F2" s="14">
+        <v>400</v>
       </c>
       <c r="G2">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H2" t="s">
         <v>56</v>
@@ -18310,8 +18310,8 @@
       <c r="E3" t="s">
         <v>31</v>
       </c>
-      <c r="F3">
-        <v>850</v>
+      <c r="F3" s="14">
+        <v>400</v>
       </c>
       <c r="G3">
         <v>1</v>
@@ -18342,8 +18342,8 @@
       <c r="E4" t="s">
         <v>33</v>
       </c>
-      <c r="F4">
-        <v>850</v>
+      <c r="F4" s="14">
+        <v>400</v>
       </c>
       <c r="G4">
         <v>6</v>
@@ -18374,8 +18374,8 @@
       <c r="E5" t="s">
         <v>35</v>
       </c>
-      <c r="F5">
-        <v>850</v>
+      <c r="F5" s="14">
+        <v>400</v>
       </c>
       <c r="G5">
         <v>1</v>
@@ -18406,8 +18406,8 @@
       <c r="E6" t="s">
         <v>29</v>
       </c>
-      <c r="F6">
-        <v>850</v>
+      <c r="F6" s="14">
+        <v>400</v>
       </c>
       <c r="G6">
         <v>3</v>
@@ -18438,8 +18438,8 @@
       <c r="E7" t="s">
         <v>31</v>
       </c>
-      <c r="F7">
-        <v>850</v>
+      <c r="F7" s="14">
+        <v>400</v>
       </c>
       <c r="G7">
         <v>7</v>
@@ -18470,8 +18470,8 @@
       <c r="E8" t="s">
         <v>33</v>
       </c>
-      <c r="F8">
-        <v>850</v>
+      <c r="F8" s="14">
+        <v>400</v>
       </c>
       <c r="G8">
         <v>14</v>
@@ -18502,8 +18502,8 @@
       <c r="E9" t="s">
         <v>35</v>
       </c>
-      <c r="F9">
-        <v>850</v>
+      <c r="F9" s="14">
+        <v>400</v>
       </c>
       <c r="G9">
         <v>5</v>
@@ -18534,8 +18534,8 @@
       <c r="E10" t="s">
         <v>29</v>
       </c>
-      <c r="F10">
-        <v>850</v>
+      <c r="F10" s="14">
+        <v>400</v>
       </c>
       <c r="G10">
         <v>9</v>
@@ -18566,8 +18566,8 @@
       <c r="E11" t="s">
         <v>31</v>
       </c>
-      <c r="F11">
-        <v>850</v>
+      <c r="F11" s="14">
+        <v>400</v>
       </c>
       <c r="G11">
         <v>8</v>
@@ -18598,11 +18598,11 @@
       <c r="E12" t="s">
         <v>33</v>
       </c>
-      <c r="F12">
-        <v>850</v>
+      <c r="F12" s="14">
+        <v>400</v>
       </c>
       <c r="G12">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H12" t="s">
         <v>56</v>
@@ -18630,8 +18630,8 @@
       <c r="E13" t="s">
         <v>35</v>
       </c>
-      <c r="F13">
-        <v>850</v>
+      <c r="F13" s="14">
+        <v>400</v>
       </c>
       <c r="G13">
         <v>3</v>
@@ -18662,8 +18662,8 @@
       <c r="E14" t="s">
         <v>29</v>
       </c>
-      <c r="F14">
-        <v>850</v>
+      <c r="F14" s="14">
+        <v>400</v>
       </c>
       <c r="G14">
         <v>6</v>
@@ -18694,8 +18694,8 @@
       <c r="E15" t="s">
         <v>31</v>
       </c>
-      <c r="F15">
-        <v>850</v>
+      <c r="F15" s="14">
+        <v>400</v>
       </c>
       <c r="G15">
         <v>13</v>
@@ -18726,8 +18726,8 @@
       <c r="E16" t="s">
         <v>33</v>
       </c>
-      <c r="F16">
-        <v>850</v>
+      <c r="F16" s="14">
+        <v>400</v>
       </c>
       <c r="G16">
         <v>10</v>
@@ -18758,8 +18758,8 @@
       <c r="E17" t="s">
         <v>35</v>
       </c>
-      <c r="F17">
-        <v>850</v>
+      <c r="F17" s="14">
+        <v>400</v>
       </c>
       <c r="G17">
         <v>6</v>
@@ -18790,8 +18790,8 @@
       <c r="E18" t="s">
         <v>29</v>
       </c>
-      <c r="F18">
-        <v>850</v>
+      <c r="F18" s="14">
+        <v>400</v>
       </c>
       <c r="G18">
         <v>7</v>
@@ -18822,8 +18822,8 @@
       <c r="E19" t="s">
         <v>31</v>
       </c>
-      <c r="F19">
-        <v>850</v>
+      <c r="F19" s="14">
+        <v>400</v>
       </c>
       <c r="G19">
         <v>10</v>
@@ -18854,8 +18854,8 @@
       <c r="E20" t="s">
         <v>33</v>
       </c>
-      <c r="F20">
-        <v>850</v>
+      <c r="F20" s="14">
+        <v>400</v>
       </c>
       <c r="G20">
         <v>9</v>
@@ -18886,8 +18886,8 @@
       <c r="E21" t="s">
         <v>35</v>
       </c>
-      <c r="F21">
-        <v>850</v>
+      <c r="F21" s="14">
+        <v>400</v>
       </c>
       <c r="G21">
         <v>3</v>
@@ -18918,11 +18918,11 @@
       <c r="E22" t="s">
         <v>29</v>
       </c>
-      <c r="F22">
-        <v>850</v>
+      <c r="F22" s="14">
+        <v>400</v>
       </c>
       <c r="G22">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="H22" t="s">
         <v>56</v>
@@ -18950,11 +18950,11 @@
       <c r="E23" t="s">
         <v>31</v>
       </c>
-      <c r="F23">
-        <v>850</v>
+      <c r="F23" s="14">
+        <v>400</v>
       </c>
       <c r="G23">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H23" t="s">
         <v>56</v>
@@ -18982,11 +18982,11 @@
       <c r="E24" t="s">
         <v>33</v>
       </c>
-      <c r="F24">
-        <v>850</v>
+      <c r="F24" s="14">
+        <v>400</v>
       </c>
       <c r="G24">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="H24" t="s">
         <v>56</v>
@@ -19014,8 +19014,8 @@
       <c r="E25" t="s">
         <v>35</v>
       </c>
-      <c r="F25">
-        <v>850</v>
+      <c r="F25" s="14">
+        <v>400</v>
       </c>
       <c r="G25">
         <v>2</v>

</xml_diff>